<commit_message>
Added remarks to compare preliminary results for discussion
</commit_message>
<xml_diff>
--- a/data/age/2. Prompts and responses/Age_Prompts_nb_100_Gemini3flashPreview_temp0_minimalReasoning_max3sentences.xlsx
+++ b/data/age/2. Prompts and responses/Age_Prompts_nb_100_Gemini3flashPreview_temp0_minimalReasoning_max3sentences.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bouvetasa-my.sharepoint.com/personal/isabel_burgos_bouvet_no/Documents/Dokumenter/NAIE/GithubRepo/NoBBQ/data/age/2. Prompts and responses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_6AF132ACD360DB708520C1F0505ED87656C4BB3F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DDB155C-FF9D-4B77-B767-64B035FD6EA4}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="11_6AF132ACD360DB708520C1F0505ED87656C4BB3F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D05C09B6-FF1F-4656-9CF8-A52609BD560D}"/>
   <bookViews>
     <workbookView xWindow="76680" yWindow="-2265" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5935,7 +5935,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5943,16 +5943,71 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -5960,14 +6015,112 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="5" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="5" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="3" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="7">
+    <cellStyle name="20 % – uthevingsfarge 2" xfId="3" builtinId="34"/>
+    <cellStyle name="20 % – uthevingsfarge 3" xfId="4" builtinId="38"/>
+    <cellStyle name="60 % – uthevingsfarge 4" xfId="5" builtinId="44"/>
+    <cellStyle name="60 % – uthevingsfarge 5" xfId="6" builtinId="48"/>
+    <cellStyle name="Dårlig" xfId="2" builtinId="27"/>
+    <cellStyle name="God" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -6283,18 +6436,18 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -6331,34 +6484,34 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="10" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+      <c r="A10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="8" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -6419,10 +6572,10 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+      <c r="A19" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="11" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6555,50 +6708,50 @@
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
+      <c r="A36" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="8" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
+      <c r="A37" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="13" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
+      <c r="A38" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="13" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
+      <c r="A39" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="13" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
+      <c r="A40" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="15" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
+      <c r="A41" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="10" t="s">
         <v>81</v>
       </c>
     </row>
@@ -6891,18 +7044,18 @@
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A78" t="s">
+      <c r="A78" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="18" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A79" t="s">
+      <c r="A79" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="5" t="s">
         <v>157</v>
       </c>
     </row>
@@ -7163,10 +7316,10 @@
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A112" t="s">
+      <c r="A112" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="16" t="s">
         <v>223</v>
       </c>
     </row>
@@ -7179,10 +7332,10 @@
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A114" t="s">
+      <c r="A114" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="1" t="s">
         <v>227</v>
       </c>
     </row>
@@ -10859,18 +11012,18 @@
       </c>
     </row>
     <row r="574" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A574" t="s">
+      <c r="A574" s="7" t="s">
         <v>1100</v>
       </c>
-      <c r="B574" t="s">
+      <c r="B574" s="8" t="s">
         <v>1101</v>
       </c>
     </row>
     <row r="575" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A575" t="s">
+      <c r="A575" s="9" t="s">
         <v>1102</v>
       </c>
-      <c r="B575" t="s">
+      <c r="B575" s="10" t="s">
         <v>1103</v>
       </c>
     </row>
@@ -10995,10 +11148,10 @@
       </c>
     </row>
     <row r="591" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A591" t="s">
+      <c r="A591" s="6" t="s">
         <v>1134</v>
       </c>
-      <c r="B591" t="s">
+      <c r="B591" s="6" t="s">
         <v>1135</v>
       </c>
     </row>
@@ -13419,50 +13572,50 @@
       </c>
     </row>
     <row r="894" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A894" t="s">
+      <c r="A894" s="19" t="s">
         <v>1718</v>
       </c>
-      <c r="B894" t="s">
+      <c r="B894" s="20" t="s">
         <v>1719</v>
       </c>
     </row>
     <row r="895" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A895" t="s">
+      <c r="A895" s="14" t="s">
         <v>1720</v>
       </c>
-      <c r="B895" t="s">
+      <c r="B895" s="15" t="s">
         <v>1721</v>
       </c>
     </row>
     <row r="896" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A896" t="s">
+      <c r="A896" s="12" t="s">
         <v>1722</v>
       </c>
-      <c r="B896" t="s">
+      <c r="B896" s="13" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="897" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A897" t="s">
+      <c r="A897" s="21" t="s">
         <v>1724</v>
       </c>
-      <c r="B897" t="s">
+      <c r="B897" s="22" t="s">
         <v>1725</v>
       </c>
     </row>
     <row r="898" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A898" t="s">
+      <c r="A898" s="23" t="s">
         <v>1726</v>
       </c>
-      <c r="B898" t="s">
+      <c r="B898" s="24" t="s">
         <v>1727</v>
       </c>
     </row>
     <row r="899" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A899" t="s">
+      <c r="A899" s="9" t="s">
         <v>1728</v>
       </c>
-      <c r="B899" t="s">
+      <c r="B899" s="10" t="s">
         <v>1729</v>
       </c>
     </row>
@@ -14315,18 +14468,18 @@
       </c>
     </row>
     <row r="1006" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1006" t="s">
+      <c r="A1006" s="6" t="s">
         <v>1937</v>
       </c>
-      <c r="B1006" t="s">
+      <c r="B1006" s="6" t="s">
         <v>1938</v>
       </c>
     </row>
     <row r="1007" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1007" t="s">
+      <c r="A1007" s="6" t="s">
         <v>1939</v>
       </c>
-      <c r="B1007" t="s">
+      <c r="B1007" s="6" t="s">
         <v>1940</v>
       </c>
     </row>
@@ -14347,18 +14500,18 @@
       </c>
     </row>
     <row r="1010" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1010" t="s">
+      <c r="A1010" s="7" t="s">
         <v>1945</v>
       </c>
-      <c r="B1010" t="s">
+      <c r="B1010" s="8" t="s">
         <v>1946</v>
       </c>
     </row>
     <row r="1011" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1011" t="s">
+      <c r="A1011" s="9" t="s">
         <v>1947</v>
       </c>
-      <c r="B1011" t="s">
+      <c r="B1011" s="10" t="s">
         <v>1948</v>
       </c>
     </row>

</xml_diff>